<commit_message>
Some more leetcode problem
</commit_message>
<xml_diff>
--- a/SupportFiles/DSA.xlsx
+++ b/SupportFiles/DSA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ishan\GITHUB\LEETCODE\SupportFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6119AFF7-B5F0-49A5-8E5C-280EE2701B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFB4F995-EEF6-4DA4-8296-7F0E0C9DE67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="24" yWindow="24" windowWidth="23016" windowHeight="12216" xr2:uid="{294B7E60-E2C0-4A38-8A3D-2163B9AC2649}"/>
   </bookViews>
@@ -382,7 +382,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCF5D703-E6BE-4222-AE3D-7D1F5B0408B3}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -409,6 +409,22 @@
         <v>567</v>
       </c>
     </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>438</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>